<commit_message>
Log MQTT data 2026-08-19 15:52 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-19.xlsx
+++ b/logs/raiv_tracker_2026-08-19.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,7 +469,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g1</t>
@@ -497,7 +496,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g4</t>
@@ -525,7 +523,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g2</t>
@@ -553,7 +550,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g3</t>
@@ -581,7 +577,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g6</t>
@@ -609,7 +604,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g8</t>
@@ -637,7 +631,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g9</t>
@@ -665,7 +658,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g11</t>
@@ -693,7 +685,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g12</t>
@@ -721,7 +712,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g13</t>
@@ -749,7 +739,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g17</t>
@@ -777,7 +766,6 @@
           <t>655</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g18</t>
@@ -805,7 +793,6 @@
           <t>642</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g19</t>
@@ -833,7 +820,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g21</t>
@@ -861,7 +847,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g5</t>
@@ -889,7 +874,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g7</t>
@@ -917,7 +901,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g10</t>
@@ -945,7 +928,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g14</t>
@@ -973,7 +955,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g15</t>
@@ -1001,7 +982,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g16</t>
@@ -1029,7 +1009,6 @@
           <t>12</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g22</t>
@@ -1057,7 +1036,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g23</t>
@@ -1085,7 +1063,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g25</t>
@@ -1113,7 +1090,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g26</t>
@@ -1141,7 +1117,6 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g27</t>
@@ -1169,7 +1144,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g28</t>
@@ -1197,7 +1171,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g29</t>
@@ -1225,7 +1198,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g30</t>
@@ -1253,7 +1225,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g34</t>
@@ -1281,7 +1252,6 @@
           <t>21</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g35</t>
@@ -1309,7 +1279,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g36</t>
@@ -1337,7 +1306,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g38</t>
@@ -1365,7 +1333,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g24</t>
@@ -1393,7 +1360,6 @@
           <t>34</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g31</t>
@@ -1421,7 +1387,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g32</t>
@@ -1449,7 +1414,6 @@
           <t>20</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g33</t>
@@ -1477,7 +1441,6 @@
           <t>21</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g37</t>
@@ -1505,7 +1468,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g39</t>
@@ -1533,7 +1495,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>raiv-tracker/truck-2/hmi/g40</t>
@@ -2123,6 +2084,2386 @@
         <v>2</v>
       </c>
       <c r="F61" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>655</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>642</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:50:50</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Truck 2</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>raiv-tracker/truck-2/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D101" t="b">
+        <v>0</v>
+      </c>
+      <c r="E101" t="n">
+        <v>11</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D102" t="b">
+        <v>1</v>
+      </c>
+      <c r="E102" t="n">
+        <v>11</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D103" t="b">
+        <v>0</v>
+      </c>
+      <c r="E103" t="n">
+        <v>11</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D104" t="b">
+        <v>0</v>
+      </c>
+      <c r="E104" t="n">
+        <v>11</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D105" t="b">
+        <v>0</v>
+      </c>
+      <c r="E105" t="n">
+        <v>11</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>4287</v>
+      </c>
+      <c r="E106" t="n">
+        <v>9</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>1820</v>
+      </c>
+      <c r="E107" t="n">
+        <v>9</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>2467</v>
+      </c>
+      <c r="E108" t="n">
+        <v>9</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>0.57546067237854</v>
+      </c>
+      <c r="E109" t="n">
+        <v>9</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>0.4245392978191376</v>
+      </c>
+      <c r="E110" t="n">
+        <v>9</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>655</v>
+      </c>
+      <c r="E111" t="n">
+        <v>9</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>10</v>
+      </c>
+      <c r="E112" t="n">
+        <v>9</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>642</v>
+      </c>
+      <c r="E113" t="n">
+        <v>9</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>0.9801526665687561</v>
+      </c>
+      <c r="E114" t="n">
+        <v>9</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>0.01526717562228441</v>
+      </c>
+      <c r="E115" t="n">
+        <v>9</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>9.16724967956543</v>
+      </c>
+      <c r="E116" t="n">
+        <v>9</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" t="n">
+        <v>3</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>0</v>
+      </c>
+      <c r="E118" t="n">
+        <v>3</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>0</v>
+      </c>
+      <c r="E119" t="n">
+        <v>3</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>4</v>
+      </c>
+      <c r="E120" t="n">
+        <v>3</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:00</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>10thsInches_Tie Next</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>135</v>
+      </c>
+      <c r="E121" t="n">
+        <v>2</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:11</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>desired_14in</t>
+        </is>
+      </c>
+      <c r="D122" t="b">
+        <v>0</v>
+      </c>
+      <c r="E122" t="n">
+        <v>11</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:11</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>desired_Pandral</t>
+        </is>
+      </c>
+      <c r="D123" t="b">
+        <v>1</v>
+      </c>
+      <c r="E123" t="n">
+        <v>11</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:11</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D124" t="b">
+        <v>0</v>
+      </c>
+      <c r="E124" t="n">
+        <v>11</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:51:11</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D125" t="b">
+        <v>1</v>
+      </c>
+      <c r="E125" t="n">
+        <v>11</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D126" t="b">
+        <v>0</v>
+      </c>
+      <c r="E126" t="n">
+        <v>11</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D127" t="b">
+        <v>1</v>
+      </c>
+      <c r="E127" t="n">
+        <v>11</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D128" t="b">
+        <v>0</v>
+      </c>
+      <c r="E128" t="n">
+        <v>11</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D129" t="b">
+        <v>0</v>
+      </c>
+      <c r="E129" t="n">
+        <v>11</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D130" t="b">
+        <v>0</v>
+      </c>
+      <c r="E130" t="n">
+        <v>11</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>4287</v>
+      </c>
+      <c r="E131" t="n">
+        <v>9</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>1820</v>
+      </c>
+      <c r="E132" t="n">
+        <v>9</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>2467</v>
+      </c>
+      <c r="E133" t="n">
+        <v>9</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>0.57546067237854</v>
+      </c>
+      <c r="E134" t="n">
+        <v>9</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>0.4245392978191376</v>
+      </c>
+      <c r="E135" t="n">
+        <v>9</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>655</v>
+      </c>
+      <c r="E136" t="n">
+        <v>9</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>10</v>
+      </c>
+      <c r="E137" t="n">
+        <v>9</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>642</v>
+      </c>
+      <c r="E138" t="n">
+        <v>9</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>0.9801526665687561</v>
+      </c>
+      <c r="E139" t="n">
+        <v>9</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>0.01526717562228441</v>
+      </c>
+      <c r="E140" t="n">
+        <v>9</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>9.16724967956543</v>
+      </c>
+      <c r="E141" t="n">
+        <v>9</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" t="n">
+        <v>3</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" t="n">
+        <v>3</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" t="n">
+        <v>3</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>4</v>
+      </c>
+      <c r="E145" t="n">
+        <v>3</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-08-19T15:52:00</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>10thsInches_Tie Next</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>135</v>
+      </c>
+      <c r="E146" t="n">
+        <v>2</v>
+      </c>
+      <c r="F146" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>